<commit_message>
Fix 135150 PPD Other row formatting bug; revert Insurance Analysis month count
openpyxl's insert_rows() shifts cell data but leaves merged-cell range
definitions anchored at their old row. The template's footer label merges
(Ending Balance per GL/TB/Variance, each spanning B:D/E:G/H:J) landed on top
of newly-inserted item rows, silently blocking writes to several columns
with no error. Also apply proper data-row formatting to every row that
holds an item, not just newly-inserted ones — the template's one spare
"buffer" row was styled as a plain divider, not a real data row.

Also reverts the Insurance Analysis "Per Month" formula back to
DATEDIF(start,end,"M") (no +1) — that tab's month count isn't governed by
the ledger's own counting convention, and the +1 was overcounting a clean
one-year policy term as 13 months instead of 12.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/revlabspm/GA_Workpaper_Template.xlsx
+++ b/data/revlabspm/GA_Workpaper_Template.xlsx
@@ -3801,11 +3801,11 @@
         <v>46185</v>
       </c>
       <c r="G7" s="173">
-        <f>D7/(DATEDIF(E7,F7,"M")+1)</f>
+        <f>D7/DATEDIF(E7,F7,"M")</f>
         <v/>
       </c>
       <c r="H7" s="173">
-        <f>IF(OR(E7="",F7=""),0,IF('Summary Page'!$C$4&lt;E7,0,IF('Summary Page'!$C$4&gt;=F7,D7,MIN(DATEDIF(DATE(YEAR(E7),MONTH(E7),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E7,F7,"M")+1)*G7-IF(DAY(E7)&gt;1,G7*(DAY(E7)-1)/DAY(EOMONTH(E7,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F7),MONTH(F7),1),IF(DAY(F7)&lt;DAY(EOMONTH(F7,0)),G7*(DAY(EOMONTH(F7,0))-DAY(F7))/DAY(EOMONTH(F7,0)),0),0))))</f>
+        <f>IF(OR(E7="",F7=""),0,IF('Summary Page'!$C$4&lt;E7,0,IF('Summary Page'!$C$4&gt;=F7,D7,MIN(DATEDIF(DATE(YEAR(E7),MONTH(E7),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E7,F7+1,"M"))*G7-IF(DAY(E7)&gt;1,G7*(DAY(E7)-1)/DAY(EOMONTH(E7,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F7),MONTH(F7),1),IF(DAY(F7)&lt;DAY(EOMONTH(F7,0)),G7*(DAY(EOMONTH(F7,0))-DAY(F7))/DAY(EOMONTH(F7,0)),0),0))))</f>
         <v/>
       </c>
       <c r="I7" s="173">
@@ -3839,11 +3839,11 @@
         <v>46185</v>
       </c>
       <c r="G8" s="176">
-        <f>D8/(DATEDIF(E8,F8,"M")+1)</f>
+        <f>D8/DATEDIF(E8,F8,"M")</f>
         <v/>
       </c>
       <c r="H8" s="176">
-        <f>IF(OR(E8="",F8=""),0,IF('Summary Page'!$C$4&lt;E8,0,IF('Summary Page'!$C$4&gt;=F8,D8,MIN(DATEDIF(DATE(YEAR(E8),MONTH(E8),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E8,F8,"M")+1)*G8-IF(DAY(E8)&gt;1,G8*(DAY(E8)-1)/DAY(EOMONTH(E8,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F8),MONTH(F8),1),IF(DAY(F8)&lt;DAY(EOMONTH(F8,0)),G8*(DAY(EOMONTH(F8,0))-DAY(F8))/DAY(EOMONTH(F8,0)),0),0))))</f>
+        <f>IF(OR(E8="",F8=""),0,IF('Summary Page'!$C$4&lt;E8,0,IF('Summary Page'!$C$4&gt;=F8,D8,MIN(DATEDIF(DATE(YEAR(E8),MONTH(E8),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E8,F8+1,"M"))*G8-IF(DAY(E8)&gt;1,G8*(DAY(E8)-1)/DAY(EOMONTH(E8,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F8),MONTH(F8),1),IF(DAY(F8)&lt;DAY(EOMONTH(F8,0)),G8*(DAY(EOMONTH(F8,0))-DAY(F8))/DAY(EOMONTH(F8,0)),0),0))))</f>
         <v/>
       </c>
       <c r="I8" s="176" t="n"/>
@@ -3877,11 +3877,11 @@
         <v>46185</v>
       </c>
       <c r="G9" s="173">
-        <f>D9/(DATEDIF(E9,F9,"M")+1)</f>
+        <f>D9/DATEDIF(E9,F9,"M")</f>
         <v/>
       </c>
       <c r="H9" s="173">
-        <f>IF(OR(E9="",F9=""),0,IF('Summary Page'!$C$4&lt;E9,0,IF('Summary Page'!$C$4&gt;=F9,D9,MIN(DATEDIF(DATE(YEAR(E9),MONTH(E9),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E9,F9,"M")+1)*G9-IF(DAY(E9)&gt;1,G9*(DAY(E9)-1)/DAY(EOMONTH(E9,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F9),MONTH(F9),1),IF(DAY(F9)&lt;DAY(EOMONTH(F9,0)),G9*(DAY(EOMONTH(F9,0))-DAY(F9))/DAY(EOMONTH(F9,0)),0),0))))</f>
+        <f>IF(OR(E9="",F9=""),0,IF('Summary Page'!$C$4&lt;E9,0,IF('Summary Page'!$C$4&gt;=F9,D9,MIN(DATEDIF(DATE(YEAR(E9),MONTH(E9),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E9,F9+1,"M"))*G9-IF(DAY(E9)&gt;1,G9*(DAY(E9)-1)/DAY(EOMONTH(E9,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F9),MONTH(F9),1),IF(DAY(F9)&lt;DAY(EOMONTH(F9,0)),G9*(DAY(EOMONTH(F9,0))-DAY(F9))/DAY(EOMONTH(F9,0)),0),0))))</f>
         <v/>
       </c>
       <c r="I9" s="173">
@@ -3915,11 +3915,11 @@
         <v>46185</v>
       </c>
       <c r="G10" s="176">
-        <f>D10/(DATEDIF(E10,F10,"M")+1)</f>
+        <f>D10/DATEDIF(E10,F10,"M")</f>
         <v/>
       </c>
       <c r="H10" s="176">
-        <f>IF(OR(E10="",F10=""),0,IF('Summary Page'!$C$4&lt;E10,0,IF('Summary Page'!$C$4&gt;=F10,D10,MIN(DATEDIF(DATE(YEAR(E10),MONTH(E10),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E10,F10,"M")+1)*G10-IF(DAY(E10)&gt;1,G10*(DAY(E10)-1)/DAY(EOMONTH(E10,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F10),MONTH(F10),1),IF(DAY(F10)&lt;DAY(EOMONTH(F10,0)),G10*(DAY(EOMONTH(F10,0))-DAY(F10))/DAY(EOMONTH(F10,0)),0),0))))</f>
+        <f>IF(OR(E10="",F10=""),0,IF('Summary Page'!$C$4&lt;E10,0,IF('Summary Page'!$C$4&gt;=F10,D10,MIN(DATEDIF(DATE(YEAR(E10),MONTH(E10),1),'Summary Page'!$C$4,"M")+1,DATEDIF(E10,F10+1,"M"))*G10-IF(DAY(E10)&gt;1,G10*(DAY(E10)-1)/DAY(EOMONTH(E10,0)),0)-IF('Summary Page'!$C$4&gt;=DATE(YEAR(F10),MONTH(F10),1),IF(DAY(F10)&lt;DAY(EOMONTH(F10,0)),G10*(DAY(EOMONTH(F10,0))-DAY(F10))/DAY(EOMONTH(F10,0)),0),0))))</f>
         <v/>
       </c>
       <c r="I10" s="176">

</xml_diff>

<commit_message>
Fix 133100/211300 amount formatting, tab label, and add Prepared by to workpaper tabs
133100 Accounts Receivable - Other: E6/E7 amount cells were General format
instead of currency, and B2 read "Loan Reserve" (leftover from copying the
115600 tab) instead of the account's own name. 211300 Accounts Payable -
Other had the same E6/E7 formatting bug.

Also add "Prepared by: Ryan Walsh" to the 20 tabs that only had a generic
"Prepared: {date}" line, matching the 3 tabs that already had it. Raw-report
tabs (rebuilt from the raw Yardi/PDF export each period) and the Summary
Page / Trial Balance tabs are intentionally left as-is — they never had
this line to begin with.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/revlabspm/GA_Workpaper_Template.xlsx
+++ b/data/revlabspm/GA_Workpaper_Template.xlsx
@@ -45,7 +45,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;\(#,##0.00\);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
@@ -53,6 +53,7 @@
     <numFmt numFmtId="168" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="169" formatCode="[$-10409]m/d/yyyy"/>
     <numFmt numFmtId="170" formatCode="[$-10409]#,##0.00;\-#,##0.00"/>
+    <numFmt numFmtId="171" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="37">
     <font>
@@ -581,7 +582,7 @@
     <xf numFmtId="14" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="268">
+  <cellXfs count="269">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1256,6 +1257,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1638,7 +1640,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="E3" s="94" t="n"/>
@@ -1851,7 +1853,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="E3" s="138" t="n"/>
@@ -3693,7 +3695,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="E3" s="138" t="n"/>
@@ -4068,7 +4070,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="E3" s="138" t="n"/>
@@ -6335,7 +6337,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="138" t="n"/>
@@ -7084,7 +7086,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -7243,7 +7245,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -7436,7 +7438,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -7649,7 +7651,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -10121,7 +10123,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -10357,7 +10359,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -10591,7 +10593,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -11587,7 +11589,12 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="192" thickBot="1"/>
+    <row r="6">
+      <c r="E6" s="268" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="192" thickBot="1">
+      <c r="E7" s="268" t="n"/>
+    </row>
     <row r="8">
       <c r="B8" s="89" t="inlineStr">
         <is>
@@ -11680,7 +11687,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="F3" s="140" t="n"/>
@@ -13340,7 +13347,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="F3" s="140" t="n"/>
@@ -13483,7 +13490,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="F3" s="140" t="n"/>
@@ -14061,7 +14068,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="F3" s="140" t="n"/>
@@ -16168,7 +16175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:T43"/>
+  <dimension ref="B1:T43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2" customWidth="1" style="192" min="1" max="1"/>
@@ -17039,7 +17046,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -17590,7 +17597,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -18021,7 +18028,7 @@
     <row r="3">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="94" t="n"/>
@@ -19616,7 +19623,7 @@
     <row r="2" ht="15" customHeight="1" s="192">
       <c r="B2" s="98" t="inlineStr">
         <is>
-          <t>Loan Reserve</t>
+          <t>Accounts Receivable - Other</t>
         </is>
       </c>
       <c r="D2" s="98" t="n"/>
@@ -19625,7 +19632,7 @@
     <row r="3" ht="15" customHeight="1" s="192">
       <c r="B3" s="138" t="inlineStr">
         <is>
-          <t>revlabs  |  Period: Jan-2026  |  Prepared: 05/12/2026</t>
+          <t>revlabs  |  Period: Jan-2026  |  Prepared by: Ryan Walsh  |  05/12/2026</t>
         </is>
       </c>
       <c r="D3" s="138" t="n"/>
@@ -19654,8 +19661,12 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="192"/>
-    <row r="7" ht="15" customHeight="1" s="192" thickBot="1"/>
+    <row r="6" ht="15" customHeight="1" s="192">
+      <c r="E6" s="268" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="192" thickBot="1">
+      <c r="E7" s="268" t="n"/>
+    </row>
     <row r="8" ht="15" customHeight="1" s="192">
       <c r="B8" s="89" t="inlineStr">
         <is>

</xml_diff>